<commit_message>
Updated form with Kevin's info
</commit_message>
<xml_diff>
--- a/submissions/GroupFormation/STA380GroupForm.xlsx
+++ b/submissions/GroupFormation/STA380GroupForm.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shenqianying/Desktop/Sta380 Project/submissions/GroupFormation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Documents\STA380-Project\submissions\GroupFormation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D749E528-D259-374C-85B7-03C8F31B4837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72CF3A9-01C7-4487-8DAC-FA7BB18A854A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="740" windowWidth="23560" windowHeight="14340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4245" yWindow="4410" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
   <si>
     <t>If left blank, you will be assigned a number.</t>
   </si>
@@ -138,13 +138,22 @@
   <si>
     <t>qqianyingshen</t>
     <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>Kevin Luo</t>
+  </si>
+  <si>
+    <t>luoyu21</t>
+  </si>
+  <si>
+    <t>KevinYuChenLuo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -237,8 +246,8 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="超链接" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -455,17 +464,17 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.1640625" customWidth="1"/>
-    <col min="4" max="4" width="18.1640625" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="6" width="13.1640625" customWidth="1"/>
+    <col min="1" max="1" width="31.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:4" ht="15.75" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -473,12 +482,12 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
     </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:4" ht="15.75" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -486,67 +495,67 @@
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:4" ht="15.75" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:4" ht="15.75" customHeight="1">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:4" ht="15.75" customHeight="1">
       <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:4" ht="15.75" customHeight="1">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:4" ht="15.75" customHeight="1">
       <c r="A9" s="3"/>
     </row>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:4" ht="15.75" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:4" ht="15.75" customHeight="1">
       <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:4" ht="15.75" customHeight="1">
       <c r="A12" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:4" ht="15.75" customHeight="1">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:4" ht="15.75" customHeight="1">
       <c r="A14" s="3"/>
     </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:4" ht="15.75" customHeight="1">
       <c r="A15" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:4" ht="15.75" customHeight="1">
       <c r="A16" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:6" ht="15.75" customHeight="1">
       <c r="A17" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:6" ht="15.75" customHeight="1">
       <c r="A18" s="3"/>
     </row>
-    <row r="20" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:6" ht="15.75" customHeight="1">
       <c r="A20" s="1"/>
       <c r="B20" s="3" t="s">
         <v>8</v>
@@ -564,7 +573,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:6" ht="15.75" customHeight="1">
       <c r="A21" s="3" t="s">
         <v>13</v>
       </c>
@@ -584,7 +593,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:6" ht="15.75" customHeight="1">
       <c r="A22" s="3" t="s">
         <v>15</v>
       </c>
@@ -604,7 +613,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:6" ht="15.75" customHeight="1">
       <c r="A23" s="3" t="s">
         <v>20</v>
       </c>
@@ -624,32 +633,47 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:6" ht="15.75" customHeight="1">
       <c r="A24" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24">
+        <v>1008166100</v>
+      </c>
+      <c r="E24" t="s">
+        <v>35</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15.75" customHeight="1">
       <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:6" ht="15.75" customHeight="1">
       <c r="A27" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:6" ht="15.75" customHeight="1">
       <c r="A28" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:6" ht="15.75" customHeight="1">
       <c r="A29" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1">
       <c r="A30" s="5" t="s">
         <v>26</v>
       </c>
@@ -658,6 +682,7 @@
   <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="F21" r:id="rId1" xr:uid="{160CEE8E-A216-BA42-91E8-BA7CDE37079B}"/>
+    <hyperlink ref="F24" r:id="rId2" xr:uid="{A4FF2D33-40A0-4420-8059-6D6845E20ADE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>